<commit_message>
edited map/wq code for report figs
</commit_message>
<xml_diff>
--- a/Data/tabular/YBLTE_sites.xlsx
+++ b/Data/tabular/YBLTE_sites.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kristinn\Downloads\coding\YBLTE\Data\tabular\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A33A4020-F7F8-4194-ACC0-611C8392563C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7984FEED-33E1-414B-90B7-C850EFD3572E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30000" yWindow="990" windowWidth="21600" windowHeight="12525" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="88">
   <si>
     <t>Rowid</t>
   </si>
@@ -281,9 +281,6 @@
     <t>YBT</t>
   </si>
   <si>
-    <t>Yolo Flyaway Farms</t>
-  </si>
-  <si>
     <t>Yolo Bypass at Tule Pond</t>
   </si>
   <si>
@@ -302,7 +299,7 @@
     <t>outsource</t>
   </si>
   <si>
-    <t>K estimated from google earth… ask Eric for station</t>
+    <t>Yolo Flyway Farms</t>
   </si>
 </sst>
 </file>
@@ -1276,7 +1273,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1314,7 +1311,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1352,7 +1349,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1390,7 +1387,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1428,7 +1425,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1466,7 +1463,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1504,7 +1501,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1542,7 +1539,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1580,7 +1577,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1618,7 +1615,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1656,12 +1653,12 @@
         <v>73</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C27" t="s">
         <v>75</v>
       </c>
       <c r="D27" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E27" t="s">
         <v>14</v>
@@ -1673,15 +1670,15 @@
         <v>-121.66727</v>
       </c>
       <c r="L27" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C28" t="s">
         <v>76</v>
       </c>
       <c r="D28" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E28" t="s">
         <v>14</v>
@@ -1693,15 +1690,15 @@
         <v>-121.72535000000001</v>
       </c>
       <c r="L28" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C29" t="s">
         <v>77</v>
       </c>
       <c r="D29" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E29" t="s">
         <v>14</v>
@@ -1713,15 +1710,15 @@
         <v>-121.80714999999999</v>
       </c>
       <c r="L29" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C30" t="s">
         <v>78</v>
       </c>
       <c r="D30" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E30" t="s">
         <v>14</v>
@@ -1733,38 +1730,35 @@
         <v>-121.92453</v>
       </c>
       <c r="L30" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C31" t="s">
         <v>79</v>
       </c>
       <c r="D31" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="E31" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="J31">
-        <v>38.367494399999998</v>
+        <v>38.360734999999998</v>
       </c>
       <c r="K31">
-        <v>-121.6367</v>
+        <v>-121.640771</v>
       </c>
       <c r="L31" t="s">
-        <v>87</v>
-      </c>
-      <c r="M31" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C32" t="s">
         <v>80</v>
       </c>
       <c r="D32" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E32" t="s">
         <v>19</v>
@@ -1776,7 +1770,7 @@
         <v>-121.63525</v>
       </c>
       <c r="L32" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>